<commit_message>
Add migration code for CHANCE-2
</commit_message>
<xml_diff>
--- a/RCA_StudyManagementSystem.Client/wwwroot/chance-2-cases.xlsx
+++ b/RCA_StudyManagementSystem.Client/wwwroot/chance-2-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RCA\Remote Files\Migration Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RCA\Repos\RCA_StudyManagementSystem\RCA_StudyManagementSystem.Client\wwwroot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04070E07-767E-4799-87A1-6F491A2A9700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FD4CD1-EA62-4789-A05C-FCE576DF99AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3090" yWindow="435" windowWidth="25710" windowHeight="15045" xr2:uid="{B4E2C1D0-C2AF-4C34-B7F7-B24C1EA1FF81}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="249">
   <si>
     <t>CCRNo</t>
   </si>
@@ -164,9 +164,6 @@
     <t>NC</t>
   </si>
   <si>
-    <t>37119</t>
-  </si>
-  <si>
     <t>09/11/1966</t>
   </si>
   <si>
@@ -236,9 +233,6 @@
     <t>Noelle</t>
   </si>
   <si>
-    <t>37025</t>
-  </si>
-  <si>
     <t>07/16/1979</t>
   </si>
   <si>
@@ -272,9 +266,6 @@
     <t>Jr</t>
   </si>
   <si>
-    <t>37049</t>
-  </si>
-  <si>
     <t>06/24/1953</t>
   </si>
   <si>
@@ -332,9 +323,6 @@
     <t>R</t>
   </si>
   <si>
-    <t>37157</t>
-  </si>
-  <si>
     <t>02/22/1951</t>
   </si>
   <si>
@@ -347,9 +335,6 @@
     <t>J</t>
   </si>
   <si>
-    <t>37081</t>
-  </si>
-  <si>
     <t>11/03/1942</t>
   </si>
   <si>
@@ -362,9 +347,6 @@
     <t>K</t>
   </si>
   <si>
-    <t>37067</t>
-  </si>
-  <si>
     <t>05/23/1945</t>
   </si>
   <si>
@@ -392,9 +374,6 @@
     <t>Sharad</t>
   </si>
   <si>
-    <t>37179</t>
-  </si>
-  <si>
     <t>10/12/1956</t>
   </si>
   <si>
@@ -407,9 +386,6 @@
     <t>Michele</t>
   </si>
   <si>
-    <t>37159</t>
-  </si>
-  <si>
     <t>04/19/1963</t>
   </si>
   <si>
@@ -449,9 +425,6 @@
     <t>Peter</t>
   </si>
   <si>
-    <t>37127</t>
-  </si>
-  <si>
     <t>01/07/1946</t>
   </si>
   <si>
@@ -464,9 +437,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>37107</t>
-  </si>
-  <si>
     <t>07/23/1958</t>
   </si>
   <si>
@@ -479,9 +449,6 @@
     <t>Best</t>
   </si>
   <si>
-    <t>37191</t>
-  </si>
-  <si>
     <t>07/10/1957</t>
   </si>
   <si>
@@ -497,9 +464,6 @@
     <t>E</t>
   </si>
   <si>
-    <t>37129</t>
-  </si>
-  <si>
     <t>12/15/1970</t>
   </si>
   <si>
@@ -509,9 +473,6 @@
     <t>Ronald</t>
   </si>
   <si>
-    <t>37133</t>
-  </si>
-  <si>
     <t>03/17/1951</t>
   </si>
   <si>
@@ -536,9 +497,6 @@
     <t>Ray</t>
   </si>
   <si>
-    <t>37101</t>
-  </si>
-  <si>
     <t>04/29/1952</t>
   </si>
   <si>
@@ -558,9 +516,6 @@
   </si>
   <si>
     <t>Wayne</t>
-  </si>
-  <si>
-    <t>37065</t>
   </si>
   <si>
     <t>04/24/1952</t>
@@ -1429,7 +1384,7 @@
         <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>38</v>
@@ -1444,7 +1399,7 @@
         <v>40</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>40</v>
@@ -1453,7 +1408,7 @@
         <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>41</v>
@@ -1461,17 +1416,17 @@
       <c r="L2" s="3">
         <v>27510</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="3">
+        <v>37135</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="Q2" s="2">
         <v>2</v>
@@ -1480,10 +1435,10 @@
         <v>1</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="U2" s="2" t="b">
         <v>0</v>
@@ -1495,7 +1450,7 @@
         <v>45618</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y2" s="7"/>
       <c r="Z2" s="2" t="b">
@@ -1508,7 +1463,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AF2" s="7"/>
       <c r="AG2" s="2">
@@ -1518,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="AI2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AJ2" s="7"/>
       <c r="AK2" s="3" t="s">
@@ -1533,14 +1488,14 @@
         <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="E3" s="3" t="s">
         <v>40</v>
       </c>
@@ -1548,7 +1503,7 @@
         <v>40</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>40</v>
@@ -1557,7 +1512,7 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>41</v>
@@ -1565,17 +1520,17 @@
       <c r="L3" s="3">
         <v>27510</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>42</v>
+      <c r="M3" s="3">
+        <v>37135</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="Q3" s="2">
         <v>2</v>
@@ -1584,7 +1539,7 @@
         <v>1</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="T3" s="3" t="s">
         <v>40</v>
@@ -1599,7 +1554,7 @@
         <v>43446</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y3" s="6">
         <v>43440</v>
@@ -1616,7 +1571,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AF3" s="7"/>
       <c r="AG3" s="2">
@@ -1626,7 +1581,7 @@
         <v>0</v>
       </c>
       <c r="AI3" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ3" s="7"/>
       <c r="AK3" s="3" t="s">
@@ -1641,10 +1596,10 @@
         <v>50</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>40</v>
@@ -1656,7 +1611,7 @@
         <v>40</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>40</v>
@@ -1665,7 +1620,7 @@
         <v>40</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>41</v>
@@ -1673,17 +1628,17 @@
       <c r="L4" s="3">
         <v>27510</v>
       </c>
-      <c r="M4" s="3" t="s">
-        <v>42</v>
+      <c r="M4" s="3">
+        <v>37135</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q4" s="2">
         <v>2</v>
@@ -1692,10 +1647,10 @@
         <v>1</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="U4" s="2" t="b">
         <v>0</v>
@@ -1707,7 +1662,7 @@
         <v>43619</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Y4" s="6">
         <v>43440</v>
@@ -1724,7 +1679,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AF4" s="7"/>
       <c r="AG4" s="2">
@@ -1734,7 +1689,7 @@
         <v>0</v>
       </c>
       <c r="AI4" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ4" s="7"/>
       <c r="AK4" s="3" t="s">
@@ -1749,14 +1704,14 @@
         <v>51</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="E5" s="3" t="s">
         <v>40</v>
       </c>
@@ -1764,7 +1719,7 @@
         <v>40</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>40</v>
@@ -1773,7 +1728,7 @@
         <v>40</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>41</v>
@@ -1781,17 +1736,17 @@
       <c r="L5" s="3">
         <v>27510</v>
       </c>
-      <c r="M5" s="3" t="s">
-        <v>42</v>
+      <c r="M5" s="3">
+        <v>37135</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q5" s="2">
         <v>2</v>
@@ -1800,7 +1755,7 @@
         <v>2</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="T5" s="3" t="s">
         <v>40</v>
@@ -1815,7 +1770,7 @@
         <v>43411</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Y5" s="6">
         <v>43440</v>
@@ -1832,7 +1787,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AF5" s="7"/>
       <c r="AG5" s="2">
@@ -1842,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="AI5" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ5" s="7"/>
       <c r="AK5" s="3" t="s">
@@ -1857,14 +1812,14 @@
         <v>55</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="E6" s="3" t="s">
         <v>40</v>
       </c>
@@ -1872,7 +1827,7 @@
         <v>40</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>40</v>
@@ -1881,7 +1836,7 @@
         <v>40</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>41</v>
@@ -1889,17 +1844,17 @@
       <c r="L6" s="3">
         <v>27510</v>
       </c>
-      <c r="M6" s="3" t="s">
-        <v>66</v>
+      <c r="M6" s="3">
+        <v>37135</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Q6" s="2">
         <v>1</v>
@@ -1908,7 +1863,7 @@
         <v>2</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="T6" s="3" t="s">
         <v>40</v>
@@ -1923,7 +1878,7 @@
         <v>43475</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y6" s="6">
         <v>43475</v>
@@ -1940,7 +1895,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="AF6" s="7"/>
       <c r="AG6" s="2">
@@ -1950,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="AI6" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ6" s="7"/>
       <c r="AK6" s="3" t="s">
@@ -1965,13 +1920,13 @@
         <v>56</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>40</v>
@@ -1980,7 +1935,7 @@
         <v>40</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>40</v>
@@ -1989,7 +1944,7 @@
         <v>40</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>41</v>
@@ -1997,17 +1952,17 @@
       <c r="L7" s="3">
         <v>27510</v>
       </c>
-      <c r="M7" s="3" t="s">
-        <v>42</v>
+      <c r="M7" s="3">
+        <v>37135</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q7" s="2">
         <v>1</v>
@@ -2016,10 +1971,10 @@
         <v>1</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="U7" s="2" t="b">
         <v>0</v>
@@ -2031,7 +1986,7 @@
         <v>43482</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y7" s="6">
         <v>43440</v>
@@ -2048,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AF7" s="7"/>
       <c r="AG7" s="2">
@@ -2058,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="AI7" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ7" s="7"/>
       <c r="AK7" s="3" t="s">
@@ -2073,10 +2028,10 @@
         <v>59</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>40</v>
@@ -2088,7 +2043,7 @@
         <v>40</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>40</v>
@@ -2097,7 +2052,7 @@
         <v>40</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>41</v>
@@ -2105,17 +2060,17 @@
       <c r="L8" s="3">
         <v>27510</v>
       </c>
-      <c r="M8" s="3" t="s">
-        <v>42</v>
+      <c r="M8" s="3">
+        <v>37135</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Q8" s="2">
         <v>2</v>
@@ -2124,10 +2079,10 @@
         <v>1</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="U8" s="2" t="b">
         <v>0</v>
@@ -2139,7 +2094,7 @@
         <v>43467</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y8" s="6">
         <v>43440</v>
@@ -2156,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AF8" s="7"/>
       <c r="AG8" s="2">
@@ -2166,7 +2121,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ8" s="7"/>
       <c r="AK8" s="3" t="s">
@@ -2181,22 +2136,22 @@
         <v>62</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>40</v>
@@ -2205,7 +2160,7 @@
         <v>40</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>41</v>
@@ -2213,17 +2168,17 @@
       <c r="L9" s="3">
         <v>27510</v>
       </c>
-      <c r="M9" s="3" t="s">
-        <v>78</v>
+      <c r="M9" s="3">
+        <v>37135</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="Q9" s="2">
         <v>1</v>
@@ -2232,7 +2187,7 @@
         <v>1</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="T9" s="3" t="s">
         <v>40</v>
@@ -2247,7 +2202,7 @@
         <v>43431</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y9" s="6">
         <v>43433</v>
@@ -2264,7 +2219,7 @@
         <v>0</v>
       </c>
       <c r="AE9" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AF9" s="7"/>
       <c r="AG9" s="2">
@@ -2274,7 +2229,7 @@
         <v>0</v>
       </c>
       <c r="AI9" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ9" s="7"/>
       <c r="AK9" s="3" t="s">
@@ -2289,13 +2244,13 @@
         <v>63</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>40</v>
@@ -2304,7 +2259,7 @@
         <v>40</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>40</v>
@@ -2313,7 +2268,7 @@
         <v>40</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>41</v>
@@ -2321,17 +2276,17 @@
       <c r="L10" s="3">
         <v>27510</v>
       </c>
-      <c r="M10" s="3" t="s">
-        <v>78</v>
+      <c r="M10" s="3">
+        <v>37135</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="Q10" s="2">
         <v>1</v>
@@ -2340,7 +2295,7 @@
         <v>1</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="T10" s="3" t="s">
         <v>40</v>
@@ -2355,7 +2310,7 @@
         <v>43417</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Y10" s="6">
         <v>43433</v>
@@ -2372,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="AF10" s="7"/>
       <c r="AG10" s="2">
@@ -2382,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="AI10" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ10" s="7"/>
       <c r="AK10" s="3" t="s">
@@ -2397,13 +2352,13 @@
         <v>64</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>40</v>
@@ -2412,7 +2367,7 @@
         <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>40</v>
@@ -2421,7 +2376,7 @@
         <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>41</v>
@@ -2429,17 +2384,17 @@
       <c r="L11" s="3">
         <v>27510</v>
       </c>
-      <c r="M11" s="3" t="s">
-        <v>78</v>
+      <c r="M11" s="3">
+        <v>37135</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q11" s="2">
         <v>2</v>
@@ -2448,10 +2403,10 @@
         <v>2</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="U11" s="2" t="b">
         <v>0</v>
@@ -2463,7 +2418,7 @@
         <v>43619</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Y11" s="6">
         <v>43440</v>
@@ -2480,7 +2435,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AF11" s="7"/>
       <c r="AG11" s="2">
@@ -2490,7 +2445,7 @@
         <v>0</v>
       </c>
       <c r="AI11" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ11" s="7"/>
       <c r="AK11" s="3" t="s">
@@ -2505,22 +2460,22 @@
         <v>65</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>40</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>40</v>
@@ -2529,7 +2484,7 @@
         <v>40</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>41</v>
@@ -2537,17 +2492,17 @@
       <c r="L12" s="3">
         <v>27510</v>
       </c>
-      <c r="M12" s="3" t="s">
-        <v>78</v>
+      <c r="M12" s="3">
+        <v>37135</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="O12" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Q12" s="2">
         <v>1</v>
@@ -2556,7 +2511,7 @@
         <v>1</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="T12" s="3" t="s">
         <v>40</v>
@@ -2571,7 +2526,7 @@
         <v>43433</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y12" s="6">
         <v>43433</v>
@@ -2588,7 +2543,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="AF12" s="7"/>
       <c r="AG12" s="2">
@@ -2598,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="AI12" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ12" s="7"/>
       <c r="AK12" s="3" t="s">
@@ -2613,13 +2568,13 @@
         <v>66</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>40</v>
@@ -2628,7 +2583,7 @@
         <v>40</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>40</v>
@@ -2637,7 +2592,7 @@
         <v>40</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>41</v>
@@ -2645,17 +2600,17 @@
       <c r="L13" s="3">
         <v>27510</v>
       </c>
-      <c r="M13" s="3" t="s">
-        <v>78</v>
+      <c r="M13" s="3">
+        <v>37135</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="O13" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="Q13" s="2">
         <v>1</v>
@@ -2664,7 +2619,7 @@
         <v>2</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="T13" s="3" t="s">
         <v>40</v>
@@ -2679,7 +2634,7 @@
         <v>43441</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y13" s="6">
         <v>43441</v>
@@ -2696,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="AE13" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AF13" s="7"/>
       <c r="AG13" s="2">
@@ -2706,7 +2661,7 @@
         <v>0</v>
       </c>
       <c r="AI13" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ13" s="7"/>
       <c r="AK13" s="3" t="s">
@@ -2721,13 +2676,13 @@
         <v>70</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>40</v>
@@ -2736,7 +2691,7 @@
         <v>40</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>40</v>
@@ -2745,7 +2700,7 @@
         <v>40</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>41</v>
@@ -2753,17 +2708,17 @@
       <c r="L14" s="3">
         <v>27510</v>
       </c>
-      <c r="M14" s="3" t="s">
-        <v>98</v>
+      <c r="M14" s="3">
+        <v>37135</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="O14" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="Q14" s="2">
         <v>1</v>
@@ -2772,7 +2727,7 @@
         <v>1</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="T14" s="3" t="s">
         <v>40</v>
@@ -2787,7 +2742,7 @@
         <v>43441</v>
       </c>
       <c r="X14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y14" s="6">
         <v>43441</v>
@@ -2804,7 +2759,7 @@
         <v>0</v>
       </c>
       <c r="AE14" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="AF14" s="7"/>
       <c r="AG14" s="2">
@@ -2814,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="AI14" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ14" s="7"/>
       <c r="AK14" s="3" t="s">
@@ -2829,13 +2784,13 @@
         <v>72</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>40</v>
@@ -2844,7 +2799,7 @@
         <v>40</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>40</v>
@@ -2853,7 +2808,7 @@
         <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>41</v>
@@ -2861,17 +2816,17 @@
       <c r="L15" s="3">
         <v>27510</v>
       </c>
-      <c r="M15" s="3" t="s">
-        <v>103</v>
+      <c r="M15" s="3">
+        <v>37135</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="O15" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Q15" s="2">
         <v>1</v>
@@ -2880,7 +2835,7 @@
         <v>1</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="T15" s="3" t="s">
         <v>40</v>
@@ -2895,7 +2850,7 @@
         <v>43440</v>
       </c>
       <c r="X15" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Y15" s="6">
         <v>43440</v>
@@ -2912,7 +2867,7 @@
         <v>0</v>
       </c>
       <c r="AE15" s="4" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="AF15" s="7"/>
       <c r="AG15" s="2">
@@ -2922,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="AI15" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ15" s="7"/>
       <c r="AK15" s="3" t="s">
@@ -2937,31 +2892,31 @@
         <v>73</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>206</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>41</v>
@@ -2969,17 +2924,17 @@
       <c r="L16" s="3">
         <v>27510</v>
       </c>
-      <c r="M16" s="3" t="s">
-        <v>108</v>
+      <c r="M16" s="3">
+        <v>37135</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>40</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="Q16" s="2">
         <v>8</v>
@@ -2988,10 +2943,10 @@
         <v>1</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="U16" s="2" t="b">
         <v>0</v>
@@ -3003,7 +2958,7 @@
         <v>45961</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y16" s="6">
         <v>43433</v>
@@ -3020,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="AF16" s="7"/>
       <c r="AG16" s="2">
@@ -3030,7 +2985,7 @@
         <v>0</v>
       </c>
       <c r="AI16" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ16" s="7"/>
       <c r="AK16" s="3" t="s">
@@ -3045,13 +3000,13 @@
         <v>4966</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>40</v>
@@ -3060,7 +3015,7 @@
         <v>40</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>40</v>
@@ -3069,7 +3024,7 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K17" s="10" t="s">
         <v>41</v>
@@ -3077,15 +3032,15 @@
       <c r="L17" s="3">
         <v>27510</v>
       </c>
-      <c r="M17" s="10" t="s">
-        <v>42</v>
+      <c r="M17" s="3">
+        <v>37135</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="O17" s="10"/>
       <c r="P17" s="11" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="Q17" s="9">
         <v>1</v>
@@ -3094,7 +3049,7 @@
         <v>2</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="T17" s="10" t="s">
         <v>40</v>
@@ -3109,7 +3064,7 @@
         <v>45821</v>
       </c>
       <c r="X17" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y17" s="13">
         <v>45827</v>
@@ -3124,7 +3079,7 @@
         <v>0</v>
       </c>
       <c r="AE17" s="11" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="AF17" s="14"/>
       <c r="AG17" s="9">
@@ -3134,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ17" s="14"/>
       <c r="AK17" s="10" t="s">
@@ -3147,10 +3102,10 @@
         <v>4968</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>40</v>
@@ -3162,7 +3117,7 @@
         <v>40</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>40</v>
@@ -3171,7 +3126,7 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>41</v>
@@ -3179,15 +3134,15 @@
       <c r="L18" s="3">
         <v>27510</v>
       </c>
-      <c r="M18" s="10" t="s">
-        <v>118</v>
+      <c r="M18" s="3">
+        <v>37135</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="O18" s="10"/>
       <c r="P18" s="11" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="Q18" s="9">
         <v>9</v>
@@ -3196,7 +3151,7 @@
         <v>1</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="T18" s="10" t="s">
         <v>40</v>
@@ -3211,7 +3166,7 @@
         <v>45824</v>
       </c>
       <c r="X18" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y18" s="13">
         <v>45827</v>
@@ -3226,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="11" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="AF18" s="14"/>
       <c r="AG18" s="9">
@@ -3236,7 +3191,7 @@
         <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ18" s="14"/>
       <c r="AK18" s="10" t="s">
@@ -3251,13 +3206,13 @@
         <v>4971</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>40</v>
@@ -3266,7 +3221,7 @@
         <v>40</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>40</v>
@@ -3275,7 +3230,7 @@
         <v>40</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K19" s="10" t="s">
         <v>41</v>
@@ -3283,17 +3238,17 @@
       <c r="L19" s="3">
         <v>27510</v>
       </c>
-      <c r="M19" s="10" t="s">
-        <v>123</v>
+      <c r="M19" s="3">
+        <v>37135</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P19" s="11" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="Q19" s="9">
         <v>2</v>
@@ -3302,7 +3257,7 @@
         <v>2</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="T19" s="10" t="s">
         <v>40</v>
@@ -3317,7 +3272,7 @@
         <v>45824</v>
       </c>
       <c r="X19" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y19" s="13">
         <v>45827</v>
@@ -3332,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="AE19" s="11" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="AF19" s="14"/>
       <c r="AG19" s="9">
@@ -3342,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ19" s="14"/>
       <c r="AK19" s="10" t="s">
@@ -3355,13 +3310,13 @@
         <v>4973</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>40</v>
@@ -3370,14 +3325,14 @@
         <v>40</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="H20" s="10"/>
       <c r="I20" s="10" t="s">
         <v>40</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>41</v>
@@ -3385,17 +3340,17 @@
       <c r="L20" s="3">
         <v>27510</v>
       </c>
-      <c r="M20" s="10" t="s">
-        <v>103</v>
+      <c r="M20" s="3">
+        <v>37135</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="O20" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P20" s="11" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="Q20" s="9">
         <v>1</v>
@@ -3404,7 +3359,7 @@
         <v>2</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
       <c r="T20" s="10" t="s">
         <v>40</v>
@@ -3419,7 +3374,7 @@
         <v>45824</v>
       </c>
       <c r="X20" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y20" s="13">
         <v>45827</v>
@@ -3434,7 +3389,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="11" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="AF20" s="14"/>
       <c r="AG20" s="9">
@@ -3444,7 +3399,7 @@
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ20" s="14"/>
       <c r="AK20" s="10" t="s">
@@ -3459,22 +3414,22 @@
         <v>4974</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>40</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>40</v>
@@ -3483,7 +3438,7 @@
         <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K21" s="10" t="s">
         <v>41</v>
@@ -3491,17 +3446,17 @@
       <c r="L21" s="3">
         <v>27510</v>
       </c>
-      <c r="M21" s="10" t="s">
-        <v>103</v>
+      <c r="M21" s="3">
+        <v>37135</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="O21" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P21" s="11" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="Q21" s="9">
         <v>1</v>
@@ -3510,10 +3465,10 @@
         <v>1</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
       <c r="T21" s="10" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="U21" s="9" t="b">
         <v>0</v>
@@ -3525,7 +3480,7 @@
         <v>45826</v>
       </c>
       <c r="X21" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y21" s="14"/>
       <c r="Z21" s="9" t="b">
@@ -3538,7 +3493,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="11" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="AF21" s="14"/>
       <c r="AG21" s="9">
@@ -3548,7 +3503,7 @@
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AJ21" s="14"/>
       <c r="AK21" s="10" t="s">
@@ -3563,13 +3518,13 @@
         <v>4975</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>40</v>
@@ -3578,7 +3533,7 @@
         <v>40</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>40</v>
@@ -3587,7 +3542,7 @@
         <v>40</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K22" s="10" t="s">
         <v>41</v>
@@ -3595,17 +3550,17 @@
       <c r="L22" s="3">
         <v>27510</v>
       </c>
-      <c r="M22" s="10" t="s">
-        <v>137</v>
+      <c r="M22" s="3">
+        <v>37135</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="O22" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P22" s="11" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="Q22" s="9">
         <v>1</v>
@@ -3614,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="T22" s="10" t="s">
         <v>40</v>
@@ -3629,7 +3584,7 @@
         <v>45824</v>
       </c>
       <c r="X22" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y22" s="13">
         <v>45827</v>
@@ -3644,7 +3599,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="11" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="AF22" s="14"/>
       <c r="AG22" s="9">
@@ -3654,7 +3609,7 @@
         <v>0</v>
       </c>
       <c r="AI22" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ22" s="14"/>
       <c r="AK22" s="10" t="s">
@@ -3667,13 +3622,13 @@
         <v>4976</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>40</v>
@@ -3682,7 +3637,7 @@
         <v>40</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>40</v>
@@ -3691,7 +3646,7 @@
         <v>40</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K23" s="10" t="s">
         <v>41</v>
@@ -3699,17 +3654,17 @@
       <c r="L23" s="3">
         <v>27510</v>
       </c>
-      <c r="M23" s="10" t="s">
-        <v>142</v>
+      <c r="M23" s="3">
+        <v>37135</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="O23" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P23" s="11" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="Q23" s="9">
         <v>1</v>
@@ -3718,7 +3673,7 @@
         <v>2</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>256</v>
+        <v>241</v>
       </c>
       <c r="T23" s="10" t="s">
         <v>40</v>
@@ -3733,7 +3688,7 @@
         <v>45826</v>
       </c>
       <c r="X23" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y23" s="13">
         <v>45827</v>
@@ -3748,7 +3703,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="11" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="AF23" s="14"/>
       <c r="AG23" s="9">
@@ -3758,7 +3713,7 @@
         <v>0</v>
       </c>
       <c r="AI23" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ23" s="14"/>
       <c r="AK23" s="10" t="s">
@@ -3771,13 +3726,13 @@
         <v>4977</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>40</v>
@@ -3786,7 +3741,7 @@
         <v>40</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>40</v>
@@ -3795,7 +3750,7 @@
         <v>40</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K24" s="10" t="s">
         <v>41</v>
@@ -3803,17 +3758,17 @@
       <c r="L24" s="3">
         <v>27510</v>
       </c>
-      <c r="M24" s="10" t="s">
-        <v>147</v>
+      <c r="M24" s="3">
+        <v>37135</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="O24" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="Q24" s="9">
         <v>1</v>
@@ -3822,10 +3777,10 @@
         <v>2</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="T24" s="10" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="U24" s="9" t="b">
         <v>0</v>
@@ -3837,7 +3792,7 @@
         <v>45834</v>
       </c>
       <c r="X24" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y24" s="14"/>
       <c r="Z24" s="9" t="b">
@@ -3850,7 +3805,7 @@
         <v>0</v>
       </c>
       <c r="AE24" s="11" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="AF24" s="14"/>
       <c r="AG24" s="9">
@@ -3860,7 +3815,7 @@
         <v>0</v>
       </c>
       <c r="AI24" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AJ24" s="14"/>
       <c r="AK24" s="10" t="s">
@@ -3875,13 +3830,13 @@
         <v>4978</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>40</v>
@@ -3890,7 +3845,7 @@
         <v>40</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>40</v>
@@ -3899,7 +3854,7 @@
         <v>40</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>41</v>
@@ -3907,15 +3862,15 @@
       <c r="L25" s="3">
         <v>27510</v>
       </c>
-      <c r="M25" s="10" t="s">
-        <v>153</v>
+      <c r="M25" s="3">
+        <v>37135</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="O25" s="10"/>
       <c r="P25" s="11" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="Q25" s="9">
         <v>1</v>
@@ -3924,7 +3879,7 @@
         <v>1</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
       <c r="T25" s="10" t="s">
         <v>40</v>
@@ -3939,7 +3894,7 @@
         <v>45831</v>
       </c>
       <c r="X25" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y25" s="13">
         <v>45834</v>
@@ -3954,7 +3909,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="11" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="AF25" s="14"/>
       <c r="AG25" s="9">
@@ -3964,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="AI25" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ25" s="14"/>
       <c r="AK25" s="10" t="s">
@@ -3979,10 +3934,10 @@
         <v>4980</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>40</v>
@@ -3994,7 +3949,7 @@
         <v>40</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="H26" s="10" t="s">
         <v>40</v>
@@ -4003,7 +3958,7 @@
         <v>40</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>41</v>
@@ -4011,17 +3966,17 @@
       <c r="L26" s="3">
         <v>27510</v>
       </c>
-      <c r="M26" s="10" t="s">
-        <v>157</v>
+      <c r="M26" s="3">
+        <v>37135</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="O26" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="Q26" s="9">
         <v>1</v>
@@ -4030,7 +3985,7 @@
         <v>1</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="T26" s="10" t="s">
         <v>40</v>
@@ -4045,7 +4000,7 @@
         <v>45833</v>
       </c>
       <c r="X26" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y26" s="13">
         <v>45834</v>
@@ -4060,7 +4015,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="11" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="AF26" s="14"/>
       <c r="AG26" s="9">
@@ -4070,7 +4025,7 @@
         <v>0</v>
       </c>
       <c r="AI26" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ26" s="14"/>
       <c r="AK26" s="10" t="s">
@@ -4083,13 +4038,13 @@
         <v>4981</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>40</v>
@@ -4098,7 +4053,7 @@
         <v>40</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="H27" s="10" t="s">
         <v>40</v>
@@ -4107,7 +4062,7 @@
         <v>40</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>41</v>
@@ -4115,17 +4070,17 @@
       <c r="L27" s="3">
         <v>27510</v>
       </c>
-      <c r="M27" s="10" t="s">
-        <v>157</v>
+      <c r="M27" s="3">
+        <v>37135</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="Q27" s="9">
         <v>1</v>
@@ -4134,10 +4089,10 @@
         <v>1</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="T27" s="10" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="U27" s="9" t="b">
         <v>0</v>
@@ -4149,7 +4104,7 @@
         <v>45834</v>
       </c>
       <c r="X27" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y27" s="14"/>
       <c r="Z27" s="9" t="b">
@@ -4162,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="AE27" s="11" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="AF27" s="14"/>
       <c r="AG27" s="9">
@@ -4172,7 +4127,7 @@
         <v>0</v>
       </c>
       <c r="AI27" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AJ27" s="14"/>
       <c r="AK27" s="10" t="s">
@@ -4187,13 +4142,13 @@
         <v>4982</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="E28" s="10" t="s">
         <v>40</v>
@@ -4202,7 +4157,7 @@
         <v>40</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="H28" s="10" t="s">
         <v>40</v>
@@ -4211,7 +4166,7 @@
         <v>40</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K28" s="10" t="s">
         <v>41</v>
@@ -4219,17 +4174,17 @@
       <c r="L28" s="3">
         <v>27510</v>
       </c>
-      <c r="M28" s="10" t="s">
-        <v>166</v>
+      <c r="M28" s="3">
+        <v>37135</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="O28" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P28" s="11" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="Q28" s="9">
         <v>1</v>
@@ -4238,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
       <c r="T28" s="10" t="s">
         <v>40</v>
@@ -4253,7 +4208,7 @@
         <v>45833</v>
       </c>
       <c r="X28" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y28" s="13">
         <v>45834</v>
@@ -4268,7 +4223,7 @@
         <v>0</v>
       </c>
       <c r="AE28" s="11" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="AF28" s="14"/>
       <c r="AG28" s="9">
@@ -4278,7 +4233,7 @@
         <v>0</v>
       </c>
       <c r="AI28" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ28" s="14"/>
       <c r="AK28" s="10" t="s">
@@ -4291,10 +4246,10 @@
         <v>4983</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>40</v>
@@ -4306,7 +4261,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>40</v>
@@ -4315,7 +4270,7 @@
         <v>40</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K29" s="10" t="s">
         <v>41</v>
@@ -4323,17 +4278,17 @@
       <c r="L29" s="3">
         <v>27510</v>
       </c>
-      <c r="M29" s="10" t="s">
-        <v>157</v>
+      <c r="M29" s="3">
+        <v>37135</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P29" s="11" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="Q29" s="9">
         <v>1</v>
@@ -4342,7 +4297,7 @@
         <v>1</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="T29" s="10" t="s">
         <v>40</v>
@@ -4357,7 +4312,7 @@
         <v>45833</v>
       </c>
       <c r="X29" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y29" s="13">
         <v>45834</v>
@@ -4372,7 +4327,7 @@
         <v>0</v>
       </c>
       <c r="AE29" s="11" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="AF29" s="14"/>
       <c r="AG29" s="9">
@@ -4382,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="AI29" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ29" s="14"/>
       <c r="AK29" s="10" t="s">
@@ -4395,13 +4350,13 @@
         <v>4984</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>40</v>
@@ -4410,7 +4365,7 @@
         <v>40</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>40</v>
@@ -4419,7 +4374,7 @@
         <v>40</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="K30" s="10" t="s">
         <v>41</v>
@@ -4427,15 +4382,15 @@
       <c r="L30" s="3">
         <v>27510</v>
       </c>
-      <c r="M30" s="10" t="s">
-        <v>174</v>
+      <c r="M30" s="3">
+        <v>37135</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="O30" s="10"/>
       <c r="P30" s="11" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="Q30" s="9">
         <v>1</v>
@@ -4444,7 +4399,7 @@
         <v>1</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="T30" s="10" t="s">
         <v>40</v>
@@ -4459,7 +4414,7 @@
         <v>45833</v>
       </c>
       <c r="X30" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="Y30" s="13">
         <v>45834</v>
@@ -4474,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="AE30" s="11" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="AF30" s="14"/>
       <c r="AG30" s="9">
@@ -4484,7 +4439,7 @@
         <v>0</v>
       </c>
       <c r="AI30" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AJ30" s="14"/>
       <c r="AK30" s="10" t="s">

</xml_diff>